<commit_message>
chore: reorder Industries/Leveraged ETFs per spreadsheet, drop Hyperliquid notes
Industries and Leveraged ETFs card order now matches the owner's edited
market_overview_categories.xlsx. Also removes all Hyperliquid/HYPE
references (owner decision: not tracking it, no plan to revisit) and
strips the one-off 5-Year Return column from the spreadsheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/market_overview_categories.xlsx
+++ b/data/market_overview_categories.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +27,6 @@
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <i val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -56,13 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -767,12 +756,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Technology</t>
         </is>
       </c>
     </row>
@@ -784,12 +773,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>XLI</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
     </row>
@@ -801,12 +790,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>XLI</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Industrials</t>
         </is>
       </c>
     </row>
@@ -835,12 +824,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Utilities</t>
         </is>
       </c>
     </row>
@@ -852,12 +841,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XLE</t>
+          <t>XLC</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Communication Services</t>
         </is>
       </c>
     </row>
@@ -869,12 +858,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
     </row>
@@ -886,12 +875,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
     </row>
@@ -937,12 +926,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
@@ -1141,12 +1130,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SPXL</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>3x S&amp;P 500</t>
+          <t>3x Semiconductors</t>
         </is>
       </c>
     </row>
@@ -1158,12 +1147,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>SPXL</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3x Small-Cap</t>
+          <t>3x S&amp;P 500</t>
         </is>
       </c>
     </row>
@@ -1175,12 +1164,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>UDOW</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>3x Dow Jones</t>
+          <t>3x Small-Cap</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1181,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>UDOW</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3x Semiconductors</t>
+          <t>3x Dow Jones</t>
         </is>
       </c>
     </row>
@@ -1490,22 +1479,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>Note:</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Hyperliquid (HYPE) requested but excluded -- Yahoo Finance's "HYPE-USD" ticker resolves to an unrelated near-worthless token, not Hyperliquid. No clean Yahoo symbol exists for Hyperliquid as of 2026-07-10.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B64:C64"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: trim Market Overview per spreadsheet (remove XLC, XLB, US5Y, XLM)
Owner edits to market_overview_categories.xlsx: dropped Communication
Services (XLC) and Materials (XLB) from Industries, 5-Year (US5Y) from
Bonds, and Stellar (XLM) from Crypto. 61 -> 57 symbols.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/market_overview_categories.xlsx
+++ b/data/market_overview_categories.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -807,12 +807,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>XLF</t>
+          <t>XLP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
     </row>
@@ -841,12 +841,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>XLC</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Health Care</t>
         </is>
       </c>
     </row>
@@ -858,12 +858,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>XLP</t>
+          <t>XLF</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Financials</t>
         </is>
       </c>
     </row>
@@ -875,12 +875,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
     </row>
@@ -892,46 +892,46 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>XLRE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Real Estate</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Oil (WTI Crude)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Industries</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>XLRE</t>
+          <t>NG</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Natural Gas</t>
         </is>
       </c>
     </row>
@@ -943,12 +943,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Oil (WTI Crude)</t>
+          <t>Gold</t>
         </is>
       </c>
     </row>
@@ -960,12 +960,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>NG</t>
+          <t>SI</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Natural Gas</t>
+          <t>Silver</t>
         </is>
       </c>
     </row>
@@ -977,12 +977,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Gold</t>
+          <t>Platinum</t>
         </is>
       </c>
     </row>
@@ -994,46 +994,46 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SI</t>
+          <t>HG</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Copper</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>US2Y</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Platinum</t>
+          <t>2-Year</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Bonds</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HG</t>
+          <t>US10Y</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Copper</t>
+          <t>10-Year</t>
         </is>
       </c>
     </row>
@@ -1045,63 +1045,63 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>US2Y</t>
+          <t>US30Y</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2-Year</t>
+          <t>30-Year</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>US5Y</t>
+          <t>TQQQ</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>5-Year</t>
+          <t>3x Nasdaq 100</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>US10Y</t>
+          <t>SOXL</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10-Year</t>
+          <t>3x Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bonds</t>
+          <t>Leveraged ETFs</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>US30Y</t>
+          <t>SPXL</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>30-Year</t>
+          <t>3x S&amp;P 500</t>
         </is>
       </c>
     </row>
@@ -1113,12 +1113,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TQQQ</t>
+          <t>TNA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3x Nasdaq 100</t>
+          <t>3x Small-Cap</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SOXL</t>
+          <t>UDOW</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>3x Semiconductors</t>
+          <t>3x Dow Jones</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1147,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SPXL</t>
+          <t>TECL</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3x S&amp;P 500</t>
+          <t>3x Technology</t>
         </is>
       </c>
     </row>
@@ -1164,12 +1164,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TNA</t>
+          <t>QLD</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>3x Small-Cap</t>
+          <t>2x Nasdaq 100</t>
         </is>
       </c>
     </row>
@@ -1181,12 +1181,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>UDOW</t>
+          <t>SSO</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3x Dow Jones</t>
+          <t>2x S&amp;P 500</t>
         </is>
       </c>
     </row>
@@ -1198,63 +1198,63 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TECL</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>3x Technology</t>
+          <t>2x Semiconductors</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>QLD</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2x Nasdaq 100</t>
+          <t>Bitcoin</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>SSO</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2x S&amp;P 500</t>
+          <t>Ethereum</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Leveraged ETFs</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>BNB</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2x Semiconductors</t>
+          <t>Binance</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1266,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>Ripple</t>
         </is>
       </c>
     </row>
@@ -1283,12 +1283,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Solana</t>
         </is>
       </c>
     </row>
@@ -1300,12 +1300,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BNB</t>
+          <t>TRX</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Tron</t>
         </is>
       </c>
     </row>
@@ -1317,12 +1317,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>DOGE</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Ripple</t>
+          <t>Dogecoin</t>
         </is>
       </c>
     </row>
@@ -1334,12 +1334,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ZEC</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Solana</t>
+          <t>Zcash</t>
         </is>
       </c>
     </row>
@@ -1351,12 +1351,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TRX</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Tron</t>
+          <t>Cardano</t>
         </is>
       </c>
     </row>
@@ -1368,12 +1368,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>DOGE</t>
+          <t>XMR</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Dogecoin</t>
+          <t>Monero</t>
         </is>
       </c>
     </row>
@@ -1385,12 +1385,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ZEC</t>
+          <t>LTC</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Zcash</t>
+          <t>Litecoin</t>
         </is>
       </c>
     </row>
@@ -1402,78 +1402,10 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>XLM</t>
+          <t>AVAX</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
-        <is>
-          <t>Stellar</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>ADA</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Cardano</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>XMR</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Monero</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>LTC</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Litecoin</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Crypto</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>AVAX</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
         <is>
           <t>Avalanche</t>
         </is>

</xml_diff>